<commit_message>
Packing calc: mark pickup customers (star/color/tooltip) + pickup setting
</commit_message>
<xml_diff>
--- a/מאסטר הגדרות אריזה.xlsx
+++ b/מאסטר הגדרות אריזה.xlsx
@@ -612,23 +612,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="46" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="46" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -646,75 +647,80 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>בא לקחת</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
           <t>כינוי בדוח</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>סוג אריזה</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>משקל שקית
 ברירת מחדל (ק"ג)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>שקיות לארגז
 (שקית ≤400ג)</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>שקיות לארגז
 (שקית 1ק"ג)</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>יחידות
 לארגז</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>מקס ק"ג
 למיכל</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>מקס ארגזים
 למשטח</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>קטגוריה
 מיוחדת</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>סוג
 לקטגוריה</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>מקס ק"ג
 לקטגוריה</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>יחידות
 לקטגוריה</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -726,47 +732,48 @@
           <t>טבעול תעשיות מזון בע"מ 557268760 (צבר)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>צבר|טבעול</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>כלוב</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
-        <v>10</v>
-      </c>
       <c r="E4" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F4" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="n">
+      <c r="G4" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr"/>
+      <c r="I4" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="J4" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>כרוב אדום</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>חביות</t>
         </is>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="M4" s="5" t="n">
         <v>110</v>
       </c>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>חביות=כרוב אדום (110 ק"ג לחבית); כלוב=פלפלים (עד 600, שקית 10 ק"ג)</t>
         </is>
@@ -778,37 +785,38 @@
           <t>סלטי גן</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>סלטי גן</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>משטח שקיות</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
-        <v>10</v>
-      </c>
       <c r="E5" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F5" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="n">
+      <c r="G5" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="J5" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
-      <c r="K5" s="7" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="N5" s="7" t="inlineStr"/>
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>משטח שקיות 10 ק"ג עד 400</t>
         </is>
@@ -820,47 +828,48 @@
           <t>חמים וטעים 511017097</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>חמים וטעים</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>כלוב</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>10</v>
-      </c>
       <c r="E6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F6" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="n">
+      <c r="G6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>פלפל אדום</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>כלוב</t>
         </is>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="M6" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>פלפל אדום לממולאים: כלוב עד 300 כדי לא למעוך</t>
         </is>
@@ -872,35 +881,36 @@
           <t>חמים וטעים- לוי מירב (זמן קפה)</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>זמן קפה</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
-        <v>10</v>
-      </c>
       <c r="E7" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F7" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="7" t="inlineStr"/>
+      <c r="J7" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="7" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
       <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="N7" s="7" t="inlineStr"/>
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>קרטונים, שקית 10 ק"ג</t>
         </is>
@@ -912,35 +922,36 @@
           <t>סלטי מונטה קרלו</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>מונטה קרלו</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="E8" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>2</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="5" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>קרטון = 2 שקיות, כל שקית 4 ק"ג</t>
         </is>
@@ -952,37 +963,38 @@
           <t>ל.ג גל סלט בע"מ</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>סלטי גל|גל סלט</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>כלוב</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
-        <v>10</v>
-      </c>
       <c r="E9" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F9" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="n">
+      <c r="G9" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n">
         <v>600</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="J9" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="7" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -990,37 +1002,38 @@
           <t>מושיקו רחל מעדני עופר בע"מ</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>מעדני עופר</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>משטח שקיות</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
-        <v>10</v>
-      </c>
       <c r="E10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F10" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="n">
+      <c r="G10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="4" t="inlineStr"/>
+      <c r="N10" s="5" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1028,35 +1041,36 @@
           <t>עינת תעשיות מזון אגש"ח בע"מ</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>עינת</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="E11" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="F11" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F11" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="7" t="inlineStr"/>
+      <c r="J11" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J11" s="6" t="inlineStr"/>
-      <c r="K11" s="7" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr"/>
       <c r="M11" s="7" t="inlineStr"/>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="N11" s="7" t="inlineStr"/>
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>עד 50-60 קרטון במשטח</t>
         </is>
@@ -1068,35 +1082,36 @@
           <t>ביכורי שדה צפון 1994 ג.ד בע"מ</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>שדה צפון</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="E12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="F12" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F12" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="n">
+        <v>10</v>
+      </c>
       <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="n">
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="5" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="5" t="inlineStr"/>
       <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>1 ק"ג=10 לארגז; 300-400 גרם=15 לארגז</t>
         </is>
@@ -1108,35 +1123,36 @@
           <t>סלטי עמים ברדה בע"מ</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr"/>
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>סלטי עמים</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="E13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="F13" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F13" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="n">
+      <c r="I13" s="7" t="inlineStr"/>
+      <c r="J13" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J13" s="6" t="inlineStr"/>
-      <c r="K13" s="7" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr"/>
-      <c r="N13" s="6" t="inlineStr"/>
+      <c r="N13" s="7" t="inlineStr"/>
+      <c r="O13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1144,37 +1160,38 @@
           <t>מדי מעדני הים התיכון בע"מ (סלטי מיקי)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>מיקי|סלטי מיקי</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>משטח שקיות</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
-        <v>10</v>
-      </c>
       <c r="E14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F14" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="n">
+      <c r="G14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="J14" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="5" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr"/>
+      <c r="N14" s="5" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1182,43 +1199,44 @@
           <t>אלוניאל בע"מ (מקדונלס)</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr"/>
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>מקדונלד|255|256</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>יחידות</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="E15" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="F15" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>10</v>
-      </c>
       <c r="G15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="n">
+      <c r="H15" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" s="7" t="inlineStr"/>
+      <c r="J15" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>מלפפון טבעות</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr"/>
       <c r="L15" s="7" t="inlineStr"/>
-      <c r="M15" s="7" t="n">
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="N15" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>יחידות (לא ק"ג); 10 שקיות בארגז, 50 ארגז במשטח; מלפפון טבעות 20 בארגז</t>
         </is>
@@ -1230,35 +1248,36 @@
           <t>אייסמן מזון 2002 בע"מ 513318501</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>אייסמן</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="E16" s="5" t="n">
         <v>0.05</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>999</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>999</v>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="n">
+        <v>999</v>
+      </c>
       <c r="H16" s="5" t="inlineStr"/>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="n">
         <v>64</v>
       </c>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="5" t="inlineStr"/>
       <c r="M16" s="5" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>שקיות 50 גרם, 64 קרטונים במשטח (שקיות/קרטון לפי הצורך)</t>
         </is>
@@ -1270,35 +1289,36 @@
           <t>רביבים עלי דשא בע"מ (עגלת עלים)</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr"/>
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>עגלת עלים</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="E17" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="F17" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F17" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="7" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="7" t="inlineStr"/>
       <c r="M17" s="7" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
+      <c r="N17" s="7" t="inlineStr"/>
+      <c r="O17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1306,35 +1326,36 @@
           <t>תממ</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>תממ</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="E18" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>20</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="n">
+        <v>20</v>
+      </c>
       <c r="H18" s="5" t="inlineStr"/>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="5" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="5" t="inlineStr"/>
       <c r="M18" s="5" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr"/>
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>20 יחידות בקרטון, בדר"כ עד רבע משטח</t>
         </is>
@@ -1346,37 +1367,38 @@
           <t>חמוצי הבית</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr"/>
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>חמוצי הבית</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>משטח שקיות</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
-        <v>10</v>
-      </c>
       <c r="E19" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F19" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G19" s="7" t="inlineStr"/>
-      <c r="H19" s="7" t="n">
+      <c r="G19" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr"/>
+      <c r="I19" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="I19" s="7" t="n">
+      <c r="J19" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="7" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="7" t="inlineStr"/>
       <c r="M19" s="7" t="inlineStr"/>
-      <c r="N19" s="6" t="inlineStr"/>
+      <c r="N19" s="7" t="inlineStr"/>
+      <c r="O19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1384,37 +1406,38 @@
           <t>חטיפי אלקיים</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>אלקיים</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>כלוב</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n">
-        <v>10</v>
-      </c>
       <c r="E20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F20" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F20" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="n">
+      <c r="G20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="J20" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="5" t="inlineStr"/>
       <c r="M20" s="5" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="N20" s="5" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1422,35 +1445,36 @@
           <t>משה קילופים בע"מ 513626069</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr"/>
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>קילופים</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="E21" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="F21" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F21" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G21" s="7" t="inlineStr"/>
+      <c r="G21" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H21" s="7" t="inlineStr"/>
-      <c r="I21" s="7" t="n">
+      <c r="I21" s="7" t="inlineStr"/>
+      <c r="J21" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="7" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="7" t="inlineStr"/>
       <c r="M21" s="7" t="inlineStr"/>
-      <c r="N21" s="6" t="inlineStr">
+      <c r="N21" s="7" t="inlineStr"/>
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>קרטון עד 10 ק"ג, שקית 1 ק"ג</t>
         </is>
@@ -1462,37 +1486,38 @@
           <t>ניר סלטים בע"מ</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>ניר סלטים</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>כלוב</t>
         </is>
       </c>
-      <c r="D22" s="5" t="n">
-        <v>10</v>
-      </c>
       <c r="E22" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F22" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F22" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="n">
+      <c r="G22" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H22" s="5" t="inlineStr"/>
+      <c r="I22" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="J22" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="5" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="5" t="inlineStr"/>
       <c r="M22" s="5" t="inlineStr"/>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="N22" s="5" t="inlineStr"/>
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>כלוב עד 600; לחלופין קרטונים עד 50 ארגז (10 שקיות/ארגז)</t>
         </is>
@@ -1504,35 +1529,36 @@
           <t>ברכת עץ השדה א.ב בע"מ</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr"/>
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>ברכת עץ</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="E23" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="7" t="n">
+      <c r="F23" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F23" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G23" s="7" t="inlineStr"/>
+      <c r="G23" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H23" s="7" t="inlineStr"/>
-      <c r="I23" s="7" t="n">
+      <c r="I23" s="7" t="inlineStr"/>
+      <c r="J23" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
-      <c r="K23" s="7" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr"/>
       <c r="L23" s="7" t="inlineStr"/>
       <c r="M23" s="7" t="inlineStr"/>
-      <c r="N23" s="6" t="inlineStr"/>
+      <c r="N23" s="7" t="inlineStr"/>
+      <c r="O23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1540,35 +1566,36 @@
           <t>שלום שיווק פרי וירק נתניה</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>שלום שיווק</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="E24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="F24" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F24" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="n">
+        <v>10</v>
+      </c>
       <c r="H24" s="5" t="inlineStr"/>
-      <c r="I24" s="5" t="n">
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="5" t="inlineStr"/>
       <c r="M24" s="5" t="inlineStr"/>
-      <c r="N24" s="4" t="inlineStr"/>
+      <c r="N24" s="5" t="inlineStr"/>
+      <c r="O24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1576,35 +1603,36 @@
           <t>טיב וטעים 2013 הסעדה בע"מ</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr"/>
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>טיב וטעים</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="E25" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="F25" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F25" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G25" s="7" t="inlineStr"/>
+      <c r="G25" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H25" s="7" t="inlineStr"/>
-      <c r="I25" s="7" t="n">
+      <c r="I25" s="7" t="inlineStr"/>
+      <c r="J25" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J25" s="6" t="inlineStr"/>
-      <c r="K25" s="7" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr"/>
       <c r="L25" s="7" t="inlineStr"/>
       <c r="M25" s="7" t="inlineStr"/>
-      <c r="N25" s="6" t="inlineStr"/>
+      <c r="N25" s="7" t="inlineStr"/>
+      <c r="O25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1612,35 +1640,36 @@
           <t>טיב וטעים- חברת החשמל</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>טיב וטעים חברת חשמל|חברת חשמל</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D26" s="5" t="n">
+      <c r="E26" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="F26" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F26" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="n">
+        <v>10</v>
+      </c>
       <c r="H26" s="5" t="inlineStr"/>
-      <c r="I26" s="5" t="n">
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" s="5" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="5" t="inlineStr"/>
       <c r="M26" s="5" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
+      <c r="N26" s="5" t="inlineStr"/>
+      <c r="O26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1648,37 +1677,38 @@
           <t>דגים מעושנים התקווה בע"מ</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr"/>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>דגים מעושנים|התקווה</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>משטח שקיות</t>
         </is>
       </c>
-      <c r="D27" s="7" t="n">
-        <v>10</v>
-      </c>
       <c r="E27" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F27" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G27" s="7" t="inlineStr"/>
-      <c r="H27" s="7" t="n">
+      <c r="G27" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" s="7" t="inlineStr"/>
+      <c r="I27" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="I27" s="7" t="n">
+      <c r="J27" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J27" s="6" t="inlineStr"/>
-      <c r="K27" s="7" t="inlineStr"/>
+      <c r="K27" s="6" t="inlineStr"/>
       <c r="L27" s="7" t="inlineStr"/>
       <c r="M27" s="7" t="inlineStr"/>
-      <c r="N27" s="6" t="inlineStr"/>
+      <c r="N27" s="7" t="inlineStr"/>
+      <c r="O27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1686,35 +1716,36 @@
           <t>ביכורי שדה דרום 513234120</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>שדה דרום</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="E28" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="F28" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F28" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="n">
+        <v>10</v>
+      </c>
       <c r="H28" s="5" t="inlineStr"/>
-      <c r="I28" s="5" t="n">
+      <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" s="5" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="5" t="inlineStr"/>
       <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr"/>
+      <c r="N28" s="5" t="inlineStr"/>
+      <c r="O28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1722,35 +1753,36 @@
           <t>לורד סנדוויץ</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr"/>
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>לורד</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="E29" s="7" t="n">
         <v>0.12</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>70</v>
       </c>
       <c r="F29" s="7" t="n">
         <v>70</v>
       </c>
-      <c r="G29" s="7" t="inlineStr"/>
+      <c r="G29" s="7" t="n">
+        <v>70</v>
+      </c>
       <c r="H29" s="7" t="inlineStr"/>
-      <c r="I29" s="7" t="n">
+      <c r="I29" s="7" t="inlineStr"/>
+      <c r="J29" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J29" s="6" t="inlineStr"/>
-      <c r="K29" s="7" t="inlineStr"/>
+      <c r="K29" s="6" t="inlineStr"/>
       <c r="L29" s="7" t="inlineStr"/>
       <c r="M29" s="7" t="inlineStr"/>
-      <c r="N29" s="6" t="inlineStr">
+      <c r="N29" s="7" t="inlineStr"/>
+      <c r="O29" s="6" t="inlineStr">
         <is>
           <t>70 יחידות בקרטון (שקית 120 גרם); או 10 שקיות/קרטון שקית 1 ק"ג</t>
         </is>
@@ -1762,35 +1794,36 @@
           <t>תפוכן- שיווק תפו"א ומזון</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>תפוכן</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="E30" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="F30" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F30" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="n">
+        <v>10</v>
+      </c>
       <c r="H30" s="5" t="inlineStr"/>
-      <c r="I30" s="5" t="n">
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" s="5" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
       <c r="L30" s="5" t="inlineStr"/>
       <c r="M30" s="5" t="inlineStr"/>
-      <c r="N30" s="4" t="inlineStr"/>
+      <c r="N30" s="5" t="inlineStr"/>
+      <c r="O30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1798,35 +1831,36 @@
           <t>תוצרת המושב בע"מ</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr"/>
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>תוצרת המושב</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D31" s="7" t="n">
+      <c r="E31" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="7" t="n">
+      <c r="F31" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F31" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G31" s="7" t="inlineStr"/>
+      <c r="G31" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H31" s="7" t="inlineStr"/>
-      <c r="I31" s="7" t="n">
+      <c r="I31" s="7" t="inlineStr"/>
+      <c r="J31" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J31" s="6" t="inlineStr"/>
-      <c r="K31" s="7" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr"/>
       <c r="L31" s="7" t="inlineStr"/>
       <c r="M31" s="7" t="inlineStr"/>
-      <c r="N31" s="6" t="inlineStr"/>
+      <c r="N31" s="7" t="inlineStr"/>
+      <c r="O31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1834,35 +1868,36 @@
           <t>ארד הרצל בע"מ</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>ארד הרצל</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D32" s="5" t="n">
+      <c r="E32" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="5" t="n">
+      <c r="F32" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F32" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="n">
+        <v>10</v>
+      </c>
       <c r="H32" s="5" t="inlineStr"/>
-      <c r="I32" s="5" t="n">
+      <c r="I32" s="5" t="inlineStr"/>
+      <c r="J32" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="5" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
       <c r="L32" s="5" t="inlineStr"/>
       <c r="M32" s="5" t="inlineStr"/>
-      <c r="N32" s="4" t="inlineStr"/>
+      <c r="N32" s="5" t="inlineStr"/>
+      <c r="O32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -1870,35 +1905,40 @@
           <t>מרינה פטריות הגליל בע"מ</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>⭐ כן</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>מרינה</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D33" s="7" t="n">
+      <c r="E33" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="7" t="n">
+      <c r="F33" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F33" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G33" s="7" t="inlineStr"/>
+      <c r="G33" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H33" s="7" t="inlineStr"/>
-      <c r="I33" s="7" t="n">
+      <c r="I33" s="7" t="inlineStr"/>
+      <c r="J33" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J33" s="6" t="inlineStr"/>
-      <c r="K33" s="7" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr"/>
       <c r="L33" s="7" t="inlineStr"/>
       <c r="M33" s="7" t="inlineStr"/>
-      <c r="N33" s="6" t="inlineStr">
+      <c r="N33" s="7" t="inlineStr"/>
+      <c r="O33" s="6" t="inlineStr">
         <is>
           <t>באים לקחת</t>
         </is>
@@ -1910,37 +1950,42 @@
           <t>שטראוס גרופ בע"מ 557268851</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>⭐ כן</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>שטראוס</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>דולב</t>
         </is>
       </c>
-      <c r="D34" s="5" t="n">
-        <v>10</v>
-      </c>
       <c r="E34" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F34" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="F34" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G34" s="5" t="inlineStr"/>
-      <c r="H34" s="5" t="n">
+      <c r="G34" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H34" s="5" t="inlineStr"/>
+      <c r="I34" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="I34" s="5" t="n">
+      <c r="J34" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="5" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
       <c r="L34" s="5" t="inlineStr"/>
       <c r="M34" s="5" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="N34" s="5" t="inlineStr"/>
+      <c r="O34" s="4" t="inlineStr">
         <is>
           <t>דולב עד 300, שקית 10 ק"ג</t>
         </is>
@@ -1952,35 +1997,40 @@
           <t>קבוצת בנדיקט בע"מ</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>⭐ כן</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>בנדיקט</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D35" s="7" t="n">
-        <v>10</v>
-      </c>
       <c r="E35" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F35" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F35" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G35" s="7" t="inlineStr"/>
+      <c r="G35" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H35" s="7" t="inlineStr"/>
-      <c r="I35" s="7" t="n">
+      <c r="I35" s="7" t="inlineStr"/>
+      <c r="J35" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J35" s="6" t="inlineStr"/>
-      <c r="K35" s="7" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr"/>
       <c r="L35" s="7" t="inlineStr"/>
       <c r="M35" s="7" t="inlineStr"/>
-      <c r="N35" s="6" t="inlineStr">
+      <c r="N35" s="7" t="inlineStr"/>
+      <c r="O35" s="6" t="inlineStr">
         <is>
           <t>באים לקחת, שקית 10 ק"ג</t>
         </is>
@@ -1992,35 +2042,40 @@
           <t>בוניטו בע"מ 514302827</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>⭐ כן</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>בוניטו</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D36" s="5" t="n">
+      <c r="E36" s="5" t="n">
         <v>0.35</v>
-      </c>
-      <c r="E36" s="5" t="n">
-        <v>8</v>
       </c>
       <c r="F36" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="G36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="n">
+        <v>8</v>
+      </c>
       <c r="H36" s="5" t="inlineStr"/>
-      <c r="I36" s="5" t="n">
+      <c r="I36" s="5" t="inlineStr"/>
+      <c r="J36" s="5" t="n">
         <v>999</v>
       </c>
-      <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" s="5" t="inlineStr"/>
+      <c r="K36" s="4" t="inlineStr"/>
       <c r="L36" s="5" t="inlineStr"/>
       <c r="M36" s="5" t="inlineStr"/>
-      <c r="N36" s="4" t="inlineStr">
+      <c r="N36" s="5" t="inlineStr"/>
+      <c r="O36" s="4" t="inlineStr">
         <is>
           <t>קרטון קטן 8 יחידות; 2 משטחים</t>
         </is>
@@ -2032,35 +2087,40 @@
           <t>מ.מ. פרי טרי 2022 בע"מ</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>⭐ כן</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>פרי טרי</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D37" s="7" t="n">
+      <c r="E37" s="7" t="n">
         <v>1</v>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>9</v>
       </c>
       <c r="F37" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="G37" s="7" t="inlineStr"/>
+      <c r="G37" s="7" t="n">
+        <v>9</v>
+      </c>
       <c r="H37" s="7" t="inlineStr"/>
-      <c r="I37" s="7" t="n">
+      <c r="I37" s="7" t="inlineStr"/>
+      <c r="J37" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J37" s="6" t="inlineStr"/>
-      <c r="K37" s="7" t="inlineStr"/>
+      <c r="K37" s="6" t="inlineStr"/>
       <c r="L37" s="7" t="inlineStr"/>
       <c r="M37" s="7" t="inlineStr"/>
-      <c r="N37" s="6" t="inlineStr">
+      <c r="N37" s="7" t="inlineStr"/>
+      <c r="O37" s="6" t="inlineStr">
         <is>
           <t>9 קופסאות בקרטון</t>
         </is>
@@ -2072,35 +2132,40 @@
           <t>רוני יצחק תעשיות מזון (שדות בעמק)</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>⭐ כן</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>שדות בעמק</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D38" s="5" t="n">
+      <c r="E38" s="5" t="n">
         <v>0.35</v>
-      </c>
-      <c r="E38" s="5" t="n">
-        <v>8</v>
       </c>
       <c r="F38" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="G38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="n">
+        <v>8</v>
+      </c>
       <c r="H38" s="5" t="inlineStr"/>
-      <c r="I38" s="5" t="n">
+      <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="5" t="n">
         <v>999</v>
       </c>
-      <c r="J38" s="4" t="inlineStr"/>
-      <c r="K38" s="5" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr"/>
       <c r="L38" s="5" t="inlineStr"/>
       <c r="M38" s="5" t="inlineStr"/>
-      <c r="N38" s="4" t="inlineStr">
+      <c r="N38" s="5" t="inlineStr"/>
+      <c r="O38" s="4" t="inlineStr">
         <is>
           <t>קרטון קטן 8 יחידות; 2 משטחים</t>
         </is>
@@ -2112,35 +2177,36 @@
           <t>סמארה</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr"/>
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>סמארה</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>קרטונים</t>
         </is>
       </c>
-      <c r="D39" s="7" t="n">
+      <c r="E39" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E39" s="7" t="n">
+      <c r="F39" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="F39" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="G39" s="7" t="inlineStr"/>
+      <c r="G39" s="7" t="n">
+        <v>10</v>
+      </c>
       <c r="H39" s="7" t="inlineStr"/>
-      <c r="I39" s="7" t="n">
+      <c r="I39" s="7" t="inlineStr"/>
+      <c r="J39" s="7" t="n">
         <v>55</v>
       </c>
-      <c r="J39" s="6" t="inlineStr"/>
-      <c r="K39" s="7" t="inlineStr"/>
+      <c r="K39" s="6" t="inlineStr"/>
       <c r="L39" s="7" t="inlineStr"/>
       <c r="M39" s="7" t="inlineStr"/>
-      <c r="N39" s="6" t="inlineStr">
+      <c r="N39" s="7" t="inlineStr"/>
+      <c r="O39" s="6" t="inlineStr">
         <is>
           <t>נוסף אוטומטית מהדוח — נא לאמת תצורת אריזה (כרגע ברירת מחדל: קרטונים)</t>
         </is>

</xml_diff>

<commit_message>
Fix Glat Alim name (packing); Thu/Fri/Sat -> Sunday sheet (order-split)
</commit_message>
<xml_diff>
--- a/מאסטר הגדרות אריזה.xlsx
+++ b/מאסטר הגדרות אריזה.xlsx
@@ -1286,13 +1286,13 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>רביבים עלי דשא בע"מ (עגלת עלים)</t>
+          <t>רביבים עלי דשא בע"מ (גלאט עלים)</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr"/>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>עגלת עלים</t>
+          <t>גלאט עלים|עגלת עלים</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">

</xml_diff>